<commit_message>
fix: template dung email placeholder, toast canh bao khi email da ton tai
- mau-hoc-sinh.xlsx va mau-giao-vien.xlsx: thay email mau that bang placeholder (email_hocsinh@gmail.com) tranh loi 'Email da ton tai' khi upload mau chua sua
- giao-vien/hoc-sinh: tach toast warning cho email trung (da ton tai) vs toast error cho loi that su

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/mau-giao-vien.xlsx
+++ b/frontend/public/mau-giao-vien.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh sach giao vien" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,46 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00FF6600"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CC5500"/>
+        <bgColor rgb="00CC5500"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E8E8"/>
+        <bgColor rgb="00E8E8E8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +72,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,87 +461,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ho_ten</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>mat_khau</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>ten_lop</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>si_so</t>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Họ và tên GV</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Email giáo viên</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Lớp chủ nhiệm</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Sĩ số</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Nguyễn Văn An</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>gv.an@truong.edu.vn</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Okr@12345</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn An (ví dụ)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>email_giaovien@school.edu.vn</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>10A1</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>35</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Trần Thị Bình</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>gv.binh@truong.edu.vn</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Okr@12345</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>10A2</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>38</v>
+      <c r="A3" s="4" t="inlineStr"/>
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>* Dòng 2 là ví dụ tham khảo - hãy xóa và nhập dữ liệu thật từ dòng 3 trở đi</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A8:E8"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>